<commit_message>
backup estable antes sustentacion
</commit_message>
<xml_diff>
--- a/temperaturas_rellenas_promedio.xlsx
+++ b/temperaturas_rellenas_promedio.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="24334"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vivia\OneDrive\Escritorio\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Proyectos\isla-calor\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3ABDE1B-507D-40A4-B546-042C4A350483}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{97E89581-D138-4ABE-9F86-0A81809067B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -29,12 +29,15 @@
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="423" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="435" uniqueCount="33">
   <si>
     <t>Año</t>
   </si>
@@ -534,6 +537,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:R144"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
@@ -593,7 +597,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>2013</v>
       </c>
@@ -649,7 +653,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>2014</v>
       </c>
@@ -663,7 +667,7 @@
         <v>22.219086136583829</v>
       </c>
       <c r="E3">
-        <v>22.652029451943779</v>
+        <v>22.6520294519438</v>
       </c>
       <c r="F3">
         <v>22.082902544277619</v>
@@ -705,7 +709,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>2015</v>
       </c>
@@ -761,7 +765,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>2016</v>
       </c>
@@ -817,7 +821,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>2017</v>
       </c>
@@ -849,7 +853,7 @@
         <v>21.631427832992649</v>
       </c>
       <c r="K6">
-        <v>-9.7185595878136208</v>
+        <v>19.718499999999999</v>
       </c>
       <c r="L6">
         <v>20.815719907407409</v>
@@ -873,7 +877,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>2018</v>
       </c>
@@ -893,10 +897,10 @@
         <v>21.346004309751962</v>
       </c>
       <c r="G7">
-        <v>-11.23426084540951</v>
+        <v>11.2342</v>
       </c>
       <c r="H7">
-        <v>-154.82170250896061</v>
+        <v>15.482100000000001</v>
       </c>
       <c r="I7">
         <v>22.158413978494629</v>
@@ -929,12 +933,12 @@
         <v>32</v>
       </c>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>2019</v>
       </c>
       <c r="B8">
-        <v>-246.55648297491041</v>
+        <v>24.6556</v>
       </c>
       <c r="C8">
         <v>22.507938988095241</v>
@@ -943,7 +947,7 @@
         <v>21.657439516129031</v>
       </c>
       <c r="E8">
-        <v>-77.663233243469364</v>
+        <v>17.6632</v>
       </c>
       <c r="F8">
         <v>21.613797043010759</v>
@@ -952,7 +956,7 @@
         <v>23.012467592592589</v>
       </c>
       <c r="H8">
-        <v>-73.212231182795705</v>
+        <v>17.321200000000001</v>
       </c>
       <c r="I8">
         <v>23.694534050179211</v>
@@ -985,12 +989,12 @@
         <v>32</v>
       </c>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>2020</v>
       </c>
       <c r="B9">
-        <v>11.5244623655914</v>
+        <v>19.5244</v>
       </c>
       <c r="C9">
         <v>23.462147988505748</v>
@@ -1005,7 +1009,7 @@
         <v>23.456527777777779</v>
       </c>
       <c r="G9">
-        <v>-7.1566050538137507</v>
+        <v>17.156605053813699</v>
       </c>
       <c r="H9">
         <v>22.007598566308239</v>
@@ -1041,7 +1045,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>2021</v>
       </c>
@@ -1052,28 +1056,28 @@
         <v>20.093000992063491</v>
       </c>
       <c r="D10">
-        <v>-23.12931754089114</v>
+        <v>23.129317540891101</v>
       </c>
       <c r="E10">
-        <v>-20.735400490908191</v>
+        <v>20.735400490908201</v>
       </c>
       <c r="F10">
-        <v>21.71335349462365</v>
+        <v>21.7133534946237</v>
       </c>
       <c r="G10">
-        <v>7.5018148148148152</v>
+        <v>17.5018148148148</v>
       </c>
       <c r="H10">
         <v>22.58357302867384</v>
       </c>
       <c r="I10">
-        <v>6.7434888774390096</v>
+        <v>16.743488877438999</v>
       </c>
       <c r="J10">
         <v>21.861053240740741</v>
       </c>
       <c r="K10">
-        <v>11.296918076879971</v>
+        <v>17.296918076880001</v>
       </c>
       <c r="L10">
         <v>21.008495370370369</v>
@@ -1097,7 +1101,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>2022</v>
       </c>
@@ -1105,16 +1109,16 @@
         <v>21.403017473118279</v>
       </c>
       <c r="C11">
-        <v>-2.626297123015874</v>
+        <v>22.626297123015799</v>
       </c>
       <c r="D11">
-        <v>9.0179569892473133</v>
+        <v>19.017956989247299</v>
       </c>
       <c r="E11">
         <v>21.490351851851852</v>
       </c>
       <c r="F11">
-        <v>-0.57613351254480394</v>
+        <v>20.5761335125448</v>
       </c>
       <c r="G11">
         <v>20.476219907407401</v>
@@ -1153,7 +1157,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>2023</v>
       </c>
@@ -1265,7 +1269,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>2023</v>
       </c>
@@ -1377,7 +1381,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>2018</v>
       </c>
@@ -1385,7 +1389,7 @@
         <v>16.888580768454911</v>
       </c>
       <c r="C16">
-        <v>-3.2549722222222228</v>
+        <v>14.2549722222222</v>
       </c>
       <c r="D16">
         <v>15.8242773297491</v>
@@ -1433,7 +1437,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="17" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>2019</v>
       </c>
@@ -1489,7 +1493,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="18" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>2020</v>
       </c>
@@ -1500,7 +1504,7 @@
         <v>20.424331772510001</v>
       </c>
       <c r="D18">
-        <v>10.0805353456254</v>
+        <v>21.0805353456254</v>
       </c>
       <c r="E18">
         <v>20.169844529887989</v>
@@ -1545,7 +1549,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="19" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>2021</v>
       </c>
@@ -1580,7 +1584,7 @@
         <v>18.34556698028674</v>
       </c>
       <c r="L19">
-        <v>-20.4989008244488</v>
+        <v>20.4989008244488</v>
       </c>
       <c r="M19">
         <v>19.117312051971329</v>
@@ -1601,7 +1605,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="20" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>2022</v>
       </c>
@@ -1657,7 +1661,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="21" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>2023</v>
       </c>
@@ -1713,7 +1717,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="22" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A22">
         <v>2019</v>
       </c>
@@ -1769,7 +1773,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="23" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A23">
         <v>2020</v>
       </c>
@@ -1825,7 +1829,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="24" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A24">
         <v>2021</v>
       </c>
@@ -1881,7 +1885,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="25" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A25">
         <v>2022</v>
       </c>
@@ -1937,7 +1941,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="26" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A26">
         <v>2023</v>
       </c>
@@ -2049,7 +2053,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="28" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A28">
         <v>2023</v>
       </c>
@@ -2161,7 +2165,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="30" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A30">
         <v>2021</v>
       </c>
@@ -2217,7 +2221,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="31" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A31">
         <v>2022</v>
       </c>
@@ -2240,7 +2244,7 @@
         <v>16.505466007921861</v>
       </c>
       <c r="H31">
-        <v>-6.4257213810396392</v>
+        <v>16.425721381039601</v>
       </c>
       <c r="I31">
         <v>22.412915368134009</v>
@@ -2273,7 +2277,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="32" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A32">
         <v>2023</v>
       </c>
@@ -2385,7 +2389,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="34" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A34">
         <v>2019</v>
       </c>
@@ -2441,7 +2445,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="35" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A35">
         <v>2020</v>
       </c>
@@ -2497,7 +2501,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="36" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A36">
         <v>2021</v>
       </c>
@@ -2553,7 +2557,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="37" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A37">
         <v>2022</v>
       </c>
@@ -2609,7 +2613,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="38" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A38">
         <v>2023</v>
       </c>
@@ -2721,7 +2725,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="40" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A40">
         <v>2022</v>
       </c>
@@ -2738,7 +2742,7 @@
         <v>11.911868791325899</v>
       </c>
       <c r="F40">
-        <v>-33.95953993055555</v>
+        <v>13.9595399305556</v>
       </c>
       <c r="G40">
         <v>17.686497685185181</v>
@@ -2777,7 +2781,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="41" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A41">
         <v>2023</v>
       </c>
@@ -2889,7 +2893,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="43" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A43">
         <v>2013</v>
       </c>
@@ -2945,7 +2949,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="44" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A44">
         <v>2014</v>
       </c>
@@ -3001,7 +3005,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="45" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A45">
         <v>2015</v>
       </c>
@@ -3057,7 +3061,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="46" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A46">
         <v>2016</v>
       </c>
@@ -3113,7 +3117,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="47" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A47">
         <v>2017</v>
       </c>
@@ -3145,13 +3149,13 @@
         <v>20.154484065144992</v>
       </c>
       <c r="K47">
-        <v>-61.888070385859407</v>
+        <v>21.8880703858594</v>
       </c>
       <c r="L47">
-        <v>-101.7178862919681</v>
+        <v>20.717886291968</v>
       </c>
       <c r="M47">
-        <v>-762.08830001792751</v>
+        <v>22.088300017927999</v>
       </c>
       <c r="N47" t="s">
         <v>7</v>
@@ -3169,33 +3173,33 @@
         <v>32</v>
       </c>
     </row>
-    <row r="48" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A48">
         <v>2018</v>
       </c>
       <c r="B48">
-        <v>-456.69796815429459</v>
+        <v>25.697968154295001</v>
       </c>
       <c r="C48">
-        <v>-639.86659219541264</v>
+        <v>26.866592195412998</v>
       </c>
       <c r="D48">
-        <v>-445.59585797491042</v>
+        <v>25.59585797491</v>
       </c>
       <c r="E48">
-        <v>-724.01755452436203</v>
+        <v>27.017554524362001</v>
       </c>
       <c r="F48">
-        <v>-541.22898618226986</v>
+        <v>27.228986182269999</v>
       </c>
       <c r="G48">
-        <v>-613.05130674321163</v>
+        <v>24.051306743211999</v>
       </c>
       <c r="H48">
-        <v>-463.63501311352559</v>
+        <v>26.635013113526</v>
       </c>
       <c r="I48">
-        <v>-251.19235663082441</v>
+        <v>25.192356630824001</v>
       </c>
       <c r="J48">
         <v>19.2515</v>
@@ -3225,7 +3229,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="49" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A49">
         <v>2019</v>
       </c>
@@ -3281,7 +3285,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="50" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A50">
         <v>2020</v>
       </c>
@@ -3337,7 +3341,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="51" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A51">
         <v>2021</v>
       </c>
@@ -3393,12 +3397,12 @@
         <v>32</v>
       </c>
     </row>
-    <row r="52" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A52">
         <v>2022</v>
       </c>
       <c r="B52">
-        <v>8.799027777777777</v>
+        <v>18.799027777777699</v>
       </c>
       <c r="C52">
         <v>19.147155257936511</v>
@@ -3413,7 +3417,7 @@
         <v>19.894905913978501</v>
       </c>
       <c r="G52">
-        <v>13.648937500000001</v>
+        <v>18.648937499999999</v>
       </c>
       <c r="H52">
         <v>19.761317204301079</v>
@@ -3428,7 +3432,7 @@
         <v>19.053308691756271</v>
       </c>
       <c r="L52">
-        <v>15.483979166666661</v>
+        <v>16.4839791666667</v>
       </c>
       <c r="M52">
         <v>19.393054723985159</v>
@@ -3449,7 +3453,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="53" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A53">
         <v>2023</v>
       </c>
@@ -3475,7 +3479,7 @@
         <v>21.352979390681011</v>
       </c>
       <c r="I53">
-        <v>7.1871462818990421</v>
+        <v>17.187146281899</v>
       </c>
       <c r="J53">
         <v>21.878396679266292</v>
@@ -3561,7 +3565,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="55" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A55">
         <v>2013</v>
       </c>
@@ -3617,7 +3621,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="56" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A56">
         <v>2014</v>
       </c>
@@ -3673,7 +3677,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="57" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A57">
         <v>2015</v>
       </c>
@@ -3729,7 +3733,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="58" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A58">
         <v>2016</v>
       </c>
@@ -3785,7 +3789,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="59" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A59">
         <v>2017</v>
       </c>
@@ -3841,7 +3845,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="60" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A60">
         <v>2018</v>
       </c>
@@ -3879,7 +3883,7 @@
         <v>21.367455847587259</v>
       </c>
       <c r="M60">
-        <v>-54.552739621099938</v>
+        <v>24.552739621099899</v>
       </c>
       <c r="N60" t="s">
         <v>8</v>
@@ -3897,7 +3901,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="61" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A61">
         <v>2019</v>
       </c>
@@ -3905,7 +3909,7 @@
         <v>22.242804659498209</v>
       </c>
       <c r="C61">
-        <v>-151.77551835317459</v>
+        <v>21.775518353174999</v>
       </c>
       <c r="D61">
         <v>22.007800179211468</v>
@@ -3926,16 +3930,16 @@
         <v>22.800692204301079</v>
       </c>
       <c r="J61">
-        <v>-9.4987893518518458</v>
+        <v>19.498789351851801</v>
       </c>
       <c r="K61">
         <v>21.409986559139789</v>
       </c>
       <c r="L61">
-        <v>-63.304372685185193</v>
+        <v>23.3043726851852</v>
       </c>
       <c r="M61">
-        <v>-68.334401881720439</v>
+        <v>23.3344018817204</v>
       </c>
       <c r="N61" t="s">
         <v>8</v>
@@ -3953,7 +3957,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="62" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A62">
         <v>2020</v>
       </c>
@@ -4009,12 +4013,12 @@
         <v>32</v>
       </c>
     </row>
-    <row r="63" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A63">
         <v>2021</v>
       </c>
       <c r="B63">
-        <v>-41.928073674068429</v>
+        <v>21.928073674068401</v>
       </c>
       <c r="C63">
         <v>22.13429733617739</v>
@@ -4041,10 +4045,10 @@
         <v>21.71056481481482</v>
       </c>
       <c r="K63">
-        <v>10.41157034050179</v>
+        <v>18.4115703405018</v>
       </c>
       <c r="L63">
-        <v>3.0792662037037051</v>
+        <v>20.0792662037037</v>
       </c>
       <c r="M63">
         <v>20.6514247311828</v>
@@ -4065,7 +4069,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="64" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A64">
         <v>2022</v>
       </c>
@@ -4073,16 +4077,16 @@
         <v>21.278331093189959</v>
       </c>
       <c r="C64">
-        <v>-5.2790823412698424</v>
+        <v>15.279082341269801</v>
       </c>
       <c r="D64">
         <v>16.348384856630819</v>
       </c>
       <c r="E64">
-        <v>-24.746937500000001</v>
+        <v>24.746937500000001</v>
       </c>
       <c r="F64">
-        <v>10.730525520288341</v>
+        <v>21.7305255202883</v>
       </c>
       <c r="G64">
         <v>20.37268518518518</v>
@@ -4121,7 +4125,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="65" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A65">
         <v>2023</v>
       </c>
@@ -4233,7 +4237,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="67" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A67">
         <v>2019</v>
       </c>
@@ -4289,7 +4293,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="68" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A68">
         <v>2020</v>
       </c>
@@ -4345,7 +4349,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="69" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A69">
         <v>2021</v>
       </c>
@@ -4401,12 +4405,12 @@
         <v>32</v>
       </c>
     </row>
-    <row r="70" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A70">
         <v>2022</v>
       </c>
       <c r="B70">
-        <v>7.1691886200716866</v>
+        <v>17.169188620071601</v>
       </c>
       <c r="C70">
         <v>18.228589781746031</v>
@@ -4415,7 +4419,7 @@
         <v>18.441408826164871</v>
       </c>
       <c r="E70">
-        <v>-83.286173148148137</v>
+        <v>18.286173148148102</v>
       </c>
       <c r="F70">
         <v>15.761783378136199</v>
@@ -4427,7 +4431,7 @@
         <v>19.502504256272399</v>
       </c>
       <c r="I70">
-        <v>7.721299059139783</v>
+        <v>17.721299059139699</v>
       </c>
       <c r="J70">
         <v>18.61407814436922</v>
@@ -4457,7 +4461,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="71" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A71">
         <v>2023</v>
       </c>
@@ -4569,7 +4573,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="73" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A73">
         <v>2022</v>
       </c>
@@ -4625,7 +4629,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="74" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A74">
         <v>2023</v>
       </c>
@@ -4737,7 +4741,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="76" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A76">
         <v>2017</v>
       </c>
@@ -4793,7 +4797,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="77" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A77">
         <v>2018</v>
       </c>
@@ -4849,7 +4853,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="78" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A78">
         <v>2019</v>
       </c>
@@ -4857,10 +4861,10 @@
         <v>22.47675325601293</v>
       </c>
       <c r="C78">
-        <v>-42.806294146825401</v>
+        <v>21.806294146825401</v>
       </c>
       <c r="D78">
-        <v>-15.794636872759851</v>
+        <v>25.794636872759899</v>
       </c>
       <c r="E78">
         <v>21.723547916666661</v>
@@ -4869,25 +4873,25 @@
         <v>21.952971326164871</v>
       </c>
       <c r="G78">
-        <v>-281.14211967592593</v>
+        <v>23.114211967592599</v>
       </c>
       <c r="H78">
         <v>23.13418705197132</v>
       </c>
       <c r="I78">
-        <v>2.8767744175627241</v>
+        <v>22.8767744175627</v>
       </c>
       <c r="J78">
-        <v>-1.393033333333336</v>
+        <v>21.3930333333333</v>
       </c>
       <c r="K78">
-        <v>-39.540679435483867</v>
+        <v>23.540679435483899</v>
       </c>
       <c r="L78">
-        <v>-66.892938888888892</v>
+        <v>25.892938888888899</v>
       </c>
       <c r="M78">
-        <v>6.8204529569892438</v>
+        <v>26.8204529569892</v>
       </c>
       <c r="N78" t="s">
         <v>11</v>
@@ -4905,7 +4909,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="79" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A79">
         <v>2020</v>
       </c>
@@ -4913,10 +4917,10 @@
         <v>22.847633064516131</v>
       </c>
       <c r="C79">
-        <v>-23.036149447949519</v>
+        <v>23.036149447949501</v>
       </c>
       <c r="D79">
-        <v>-126.98111379928319</v>
+        <v>21.981113799283001</v>
       </c>
       <c r="E79">
         <v>22.210691435185179</v>
@@ -4928,22 +4932,22 @@
         <v>18.827550694444451</v>
       </c>
       <c r="H79">
-        <v>-17.75834363799283</v>
+        <v>17.758343637992802</v>
       </c>
       <c r="I79">
-        <v>13.468847446236561</v>
+        <v>23.468847446236602</v>
       </c>
       <c r="J79">
-        <v>2.735922222222221</v>
+        <v>22.7359222222222</v>
       </c>
       <c r="K79">
         <v>20.496387544802872</v>
       </c>
       <c r="L79">
-        <v>-2.2297879629629618</v>
+        <v>22.229787962962899</v>
       </c>
       <c r="M79">
-        <v>-24.18883042114695</v>
+        <v>24.1888304211469</v>
       </c>
       <c r="N79" t="s">
         <v>11</v>
@@ -4961,12 +4965,12 @@
         <v>32</v>
       </c>
     </row>
-    <row r="80" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A80">
         <v>2021</v>
       </c>
       <c r="B80">
-        <v>7.3246877240143382</v>
+        <v>23.3246877240143</v>
       </c>
       <c r="C80">
         <v>22.59820486111111</v>
@@ -4978,7 +4982,7 @@
         <v>22.14809305555556</v>
       </c>
       <c r="F80">
-        <v>-8.2097131657828015</v>
+        <v>18.209713165782802</v>
       </c>
       <c r="G80">
         <v>21.600689583333342</v>
@@ -4987,16 +4991,16 @@
         <v>22.94799903776762</v>
       </c>
       <c r="I80">
-        <v>-130.2459633027523</v>
+        <v>23.245963302751999</v>
       </c>
       <c r="J80">
-        <v>-55.353972123731523</v>
+        <v>25.353972123731499</v>
       </c>
       <c r="K80">
-        <v>10.93730686309738</v>
+        <v>23.937306863097401</v>
       </c>
       <c r="L80">
-        <v>-27.333054861111101</v>
+        <v>27.333054861111101</v>
       </c>
       <c r="M80">
         <v>4.7808402777777754</v>
@@ -5017,7 +5021,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="81" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A81">
         <v>2022</v>
       </c>
@@ -5034,10 +5038,10 @@
         <v>21.741413888888889</v>
       </c>
       <c r="F81">
-        <v>-45.678304450173748</v>
+        <v>25.678304450173702</v>
       </c>
       <c r="G81">
-        <v>-9.1121053240740775</v>
+        <v>19.112105324074001</v>
       </c>
       <c r="H81">
         <v>22.514681227598569</v>
@@ -5049,7 +5053,7 @@
         <v>14.37442314814815</v>
       </c>
       <c r="K81">
-        <v>-0.4489399641577082</v>
+        <v>20.448939964157699</v>
       </c>
       <c r="L81">
         <v>20.884046064814811</v>
@@ -5073,7 +5077,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="82" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A82">
         <v>2023</v>
       </c>
@@ -5241,7 +5245,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="85" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A85">
         <v>2019</v>
       </c>
@@ -5297,7 +5301,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="86" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A86">
         <v>2020</v>
       </c>
@@ -5353,7 +5357,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="87" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A87">
         <v>2021</v>
       </c>
@@ -5379,7 +5383,7 @@
         <v>21.052173720746151</v>
       </c>
       <c r="I87">
-        <v>-1.6201383058499099</v>
+        <v>21.620138305849899</v>
       </c>
       <c r="J87">
         <v>20.259136657326142</v>
@@ -5409,7 +5413,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="88" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A88">
         <v>2022</v>
       </c>
@@ -5465,7 +5469,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="89" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A89">
         <v>2023</v>
       </c>
@@ -5633,42 +5637,42 @@
         <v>32</v>
       </c>
     </row>
-    <row r="92" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A92">
         <v>2021</v>
       </c>
       <c r="B92">
-        <v>-52.01603429658384</v>
+        <v>15.016034296583801</v>
       </c>
       <c r="C92">
-        <v>-52.01603429658384</v>
+        <v>12.016034296583801</v>
       </c>
       <c r="D92">
-        <v>-52.01603429658384</v>
+        <v>12.016034296583801</v>
       </c>
       <c r="E92">
-        <v>-52.01603429658384</v>
+        <v>10.016034296583801</v>
       </c>
       <c r="F92">
-        <v>-52.01603429658384</v>
+        <v>12.016034296583801</v>
       </c>
       <c r="G92">
-        <v>-69.694948412698409</v>
+        <v>11.6949484126984</v>
       </c>
       <c r="H92">
-        <v>12.292493223110871</v>
+        <v>12.292493223110901</v>
       </c>
       <c r="I92">
-        <v>11.32197043010753</v>
+        <v>11.3219704301075</v>
       </c>
       <c r="J92">
-        <v>11.92234212962963</v>
+        <v>11.9223421296296</v>
       </c>
       <c r="K92">
         <v>11.680604390680999</v>
       </c>
       <c r="L92">
-        <v>11.50602777777778</v>
+        <v>11.506027777777801</v>
       </c>
       <c r="M92">
         <v>-353.14072961469532</v>
@@ -5689,42 +5693,42 @@
         <v>32</v>
       </c>
     </row>
-    <row r="93" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A93">
         <v>2022</v>
       </c>
       <c r="B93">
-        <v>10.827558467741939</v>
+        <v>12.8275584677419</v>
       </c>
       <c r="C93">
-        <v>11.005996775793649</v>
+        <v>11.0059967757936</v>
       </c>
       <c r="D93">
-        <v>11.33127710573477</v>
+        <v>11.331277105734801</v>
       </c>
       <c r="E93">
-        <v>8.8052950128775471</v>
+        <v>12.805295012877499</v>
       </c>
       <c r="F93">
-        <v>12.380290770609321</v>
+        <v>12.380290770609299</v>
       </c>
       <c r="G93">
-        <v>11.30612041952609</v>
+        <v>11.306120419526099</v>
       </c>
       <c r="H93">
-        <v>12.118916616219369</v>
+        <v>12.1189166162194</v>
       </c>
       <c r="I93">
-        <v>11.94121907076557</v>
+        <v>11.9412190707656</v>
       </c>
       <c r="J93">
-        <v>11.72361102106969</v>
+        <v>11.723611021069701</v>
       </c>
       <c r="K93">
-        <v>11.54941674885681</v>
+        <v>11.5494167488568</v>
       </c>
       <c r="L93">
-        <v>11.35064141496094</v>
+        <v>11.350641414960901</v>
       </c>
       <c r="M93">
         <v>11.27181920930561</v>
@@ -5745,7 +5749,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="94" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A94">
         <v>2023</v>
       </c>
@@ -5753,25 +5757,25 @@
         <v>11.6401189846642</v>
       </c>
       <c r="C94">
-        <v>11.88402977025132</v>
+        <v>11.884029770251299</v>
       </c>
       <c r="D94">
-        <v>11.45593412502801</v>
+        <v>11.455934125028</v>
       </c>
       <c r="E94">
-        <v>12.049071856287419</v>
+        <v>12.0490718562874</v>
       </c>
       <c r="F94">
-        <v>13.097731018840809</v>
+        <v>13.0977310188408</v>
       </c>
       <c r="G94">
-        <v>13.004499664204159</v>
+        <v>13.0044996642042</v>
       </c>
       <c r="H94">
-        <v>12.64195382924148</v>
+        <v>12.641953829241499</v>
       </c>
       <c r="I94">
-        <v>13.13674281553619</v>
+        <v>13.1367428155362</v>
       </c>
       <c r="J94">
         <v>13.307010283014501</v>
@@ -5857,7 +5861,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="96" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A96">
         <v>2020</v>
       </c>
@@ -5913,7 +5917,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="97" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A97">
         <v>2021</v>
       </c>
@@ -5969,7 +5973,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="98" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A98">
         <v>2022</v>
       </c>
@@ -6025,7 +6029,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="99" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A99">
         <v>2023</v>
       </c>
@@ -6137,7 +6141,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="101" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A101">
         <v>2020</v>
       </c>
@@ -6193,7 +6197,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="102" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A102">
         <v>2021</v>
       </c>
@@ -6219,7 +6223,7 @@
         <v>21.974207661290329</v>
       </c>
       <c r="I102">
-        <v>-5.8285036372453929</v>
+        <v>25.828503637245301</v>
       </c>
       <c r="J102">
         <v>21.21878634259259</v>
@@ -6249,7 +6253,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="103" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A103">
         <v>2022</v>
       </c>
@@ -6257,13 +6261,13 @@
         <v>20.846327956989249</v>
       </c>
       <c r="C103">
-        <v>-213.92942984817481</v>
+        <v>21.392942984817498</v>
       </c>
       <c r="D103">
         <v>20.620849014336919</v>
       </c>
       <c r="E103">
-        <v>-183.2081578703704</v>
+        <v>18.208157870370002</v>
       </c>
       <c r="F103">
         <v>21.34589493727599</v>
@@ -6305,7 +6309,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="104" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A104">
         <v>2023</v>
       </c>
@@ -6417,7 +6421,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="106" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A106">
         <v>2019</v>
       </c>
@@ -6473,7 +6477,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="107" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A107">
         <v>2020</v>
       </c>
@@ -6529,7 +6533,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="108" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A108">
         <v>2021</v>
       </c>
@@ -6585,7 +6589,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="109" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A109">
         <v>2022</v>
       </c>
@@ -6641,7 +6645,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="110" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A110">
         <v>2023</v>
       </c>
@@ -6753,7 +6757,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="112" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A112">
         <v>2019</v>
       </c>
@@ -6809,7 +6813,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="113" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A113">
         <v>2020</v>
       </c>
@@ -6865,7 +6869,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="114" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A114">
         <v>2021</v>
       </c>
@@ -6921,7 +6925,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="115" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A115">
         <v>2022</v>
       </c>
@@ -6977,7 +6981,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="116" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A116">
         <v>2023</v>
       </c>
@@ -7089,7 +7093,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="118" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A118">
         <v>2013</v>
       </c>
@@ -7145,7 +7149,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="119" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A119">
         <v>2014</v>
       </c>
@@ -7201,7 +7205,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="120" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A120">
         <v>2015</v>
       </c>
@@ -7257,7 +7261,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="121" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A121">
         <v>2016</v>
       </c>
@@ -7313,7 +7317,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="122" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A122">
         <v>2017</v>
       </c>
@@ -7351,7 +7355,7 @@
         <v>21.156233156769819</v>
       </c>
       <c r="M122">
-        <v>-36.436589310987813</v>
+        <v>23.436589310987799</v>
       </c>
       <c r="N122" t="s">
         <v>9</v>
@@ -7369,7 +7373,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="123" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A123">
         <v>2018</v>
       </c>
@@ -7377,13 +7381,13 @@
         <v>20.682320788530468</v>
       </c>
       <c r="C123">
-        <v>14.68413442460318</v>
+        <v>24.684134424603201</v>
       </c>
       <c r="D123">
-        <v>-5.6780017921146957</v>
+        <v>25.678001792114699</v>
       </c>
       <c r="E123">
-        <v>-13.639233185777529</v>
+        <v>23.639233185777499</v>
       </c>
       <c r="F123">
         <v>20.249146505376341</v>
@@ -7395,13 +7399,13 @@
         <v>22.21070340501792</v>
       </c>
       <c r="I123">
-        <v>-267.3556608422939</v>
+        <v>26.735566084229401</v>
       </c>
       <c r="J123">
-        <v>-51.572009259259247</v>
+        <v>18.5720092592592</v>
       </c>
       <c r="K123">
-        <v>-15.45432883830261</v>
+        <v>19.454328838302601</v>
       </c>
       <c r="L123">
         <v>21.043395833333332</v>
@@ -7425,18 +7429,18 @@
         <v>32</v>
       </c>
     </row>
-    <row r="124" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A124">
         <v>2019</v>
       </c>
       <c r="B124">
-        <v>-10.311378761736171</v>
+        <v>20.311378761736201</v>
       </c>
       <c r="C124">
-        <v>-140.0082787698413</v>
+        <v>24.008278769840999</v>
       </c>
       <c r="D124">
-        <v>-13.829912634408601</v>
+        <v>23.829912634408601</v>
       </c>
       <c r="E124">
         <v>20.603652777777771</v>
@@ -7445,7 +7449,7 @@
         <v>21.506440412186379</v>
       </c>
       <c r="G124">
-        <v>-120.5784583333333</v>
+        <v>20.578458333333</v>
       </c>
       <c r="H124">
         <v>22.53211693548387</v>
@@ -7454,13 +7458,13 @@
         <v>23.310040322580651</v>
       </c>
       <c r="J124">
-        <v>-50.36317592592593</v>
+        <v>20.363175925925901</v>
       </c>
       <c r="K124">
         <v>20.911196236559139</v>
       </c>
       <c r="L124">
-        <v>-17.7573339547891</v>
+        <v>17.7573339547891</v>
       </c>
       <c r="M124">
         <v>21.936359767025088</v>
@@ -7481,7 +7485,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="125" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A125">
         <v>2020</v>
       </c>
@@ -7537,7 +7541,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="126" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A126">
         <v>2021</v>
       </c>
@@ -7557,7 +7561,7 @@
         <v>21.309162186379929</v>
       </c>
       <c r="G126">
-        <v>-7.1031064814814817</v>
+        <v>23.103106481481401</v>
       </c>
       <c r="H126">
         <v>22.139325716845882</v>
@@ -7593,7 +7597,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="127" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A127">
         <v>2022</v>
       </c>
@@ -7649,7 +7653,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="128" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A128">
         <v>2023</v>
       </c>
@@ -7761,7 +7765,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="130" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A130">
         <v>2013</v>
       </c>
@@ -7817,7 +7821,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="131" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A131">
         <v>2014</v>
       </c>
@@ -7873,7 +7877,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="132" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A132">
         <v>2015</v>
       </c>
@@ -7929,7 +7933,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="133" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A133">
         <v>2016</v>
       </c>
@@ -7981,46 +7985,49 @@
       <c r="Q133">
         <v>6.2649999999999997</v>
       </c>
-    </row>
-    <row r="134" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="R133" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="134" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A134">
         <v>2017</v>
       </c>
       <c r="B134">
-        <v>21.57198112147432</v>
+        <v>27.571981121474298</v>
       </c>
       <c r="C134">
-        <v>22.56299023235163</v>
+        <v>27.562990232351599</v>
       </c>
       <c r="D134">
-        <v>20.898263947412779</v>
+        <v>27.898263947412801</v>
       </c>
       <c r="E134">
-        <v>22.300962768225091</v>
+        <v>27.300962768225101</v>
       </c>
       <c r="F134">
-        <v>21.869883684375981</v>
+        <v>28.869883684375999</v>
       </c>
       <c r="G134">
-        <v>21.838549880419599</v>
+        <v>28.838549880419599</v>
       </c>
       <c r="H134">
-        <v>23.042253100597151</v>
+        <v>28.0422531005972</v>
       </c>
       <c r="I134">
-        <v>22.45630404285167</v>
+        <v>28.456304042851698</v>
       </c>
       <c r="J134">
-        <v>15.59598595848596</v>
+        <v>25.595985958486001</v>
       </c>
       <c r="K134">
-        <v>12.927782258064511</v>
+        <v>27.9277822580645</v>
       </c>
       <c r="L134">
-        <v>-6.2248078703703724</v>
+        <v>26.224807870370299</v>
       </c>
       <c r="M134">
-        <v>21.474343637992831</v>
+        <v>27.474343637992799</v>
       </c>
       <c r="N134" t="s">
         <v>10</v>
@@ -8034,8 +8041,11 @@
       <c r="Q134">
         <v>6.2649999999999997</v>
       </c>
-    </row>
-    <row r="135" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="R134" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="135" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A135">
         <v>2018</v>
       </c>
@@ -8043,7 +8053,7 @@
         <v>21.023405017921149</v>
       </c>
       <c r="C135">
-        <v>15.12025793650794</v>
+        <v>21.120257936507901</v>
       </c>
       <c r="D135">
         <v>22.164881272401431</v>
@@ -8052,19 +8062,19 @@
         <v>21.294152777777779</v>
       </c>
       <c r="F135">
-        <v>-16.248259534169449</v>
+        <v>16.248259534169399</v>
       </c>
       <c r="G135">
-        <v>-99.693437500000002</v>
+        <v>19.693437500000002</v>
       </c>
       <c r="H135">
-        <v>-38.695035842293898</v>
+        <v>18.695035842293901</v>
       </c>
       <c r="I135">
-        <v>-395.13065636200719</v>
+        <v>19.130656362006999</v>
       </c>
       <c r="J135">
-        <v>13.348930555555549</v>
+        <v>18.348930555555501</v>
       </c>
       <c r="K135">
         <v>19.808705197132621</v>
@@ -8073,7 +8083,7 @@
         <v>18.184400462962969</v>
       </c>
       <c r="M135">
-        <v>13.46167501853891</v>
+        <v>15.4616750185389</v>
       </c>
       <c r="N135" t="s">
         <v>10</v>
@@ -8087,8 +8097,11 @@
       <c r="Q135">
         <v>6.2649999999999997</v>
       </c>
-    </row>
-    <row r="136" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="R135" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="136" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A136">
         <v>2019</v>
       </c>
@@ -8096,7 +8109,7 @@
         <v>22.290681003584229</v>
       </c>
       <c r="C136">
-        <v>1.070062003968252</v>
+        <v>21.0700620039682</v>
       </c>
       <c r="D136">
         <v>21.981610663082439</v>
@@ -8114,7 +8127,7 @@
         <v>22.953064516129029</v>
       </c>
       <c r="I136">
-        <v>14.187018369175631</v>
+        <v>24.1870183691756</v>
       </c>
       <c r="J136">
         <v>22.683768518518519</v>
@@ -8123,10 +8136,10 @@
         <v>18.009068100358419</v>
       </c>
       <c r="L136">
-        <v>-137.2511022044088</v>
+        <v>17.251102204409001</v>
       </c>
       <c r="M136">
-        <v>27.6</v>
+        <v>27.622299999999999</v>
       </c>
       <c r="N136" t="s">
         <v>10</v>
@@ -8140,31 +8153,34 @@
       <c r="Q136">
         <v>6.2649999999999997</v>
       </c>
-    </row>
-    <row r="137" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="R136" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="137" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A137">
         <v>2020</v>
       </c>
       <c r="B137">
-        <v>12.262876369845291</v>
+        <v>21.262876369845301</v>
       </c>
       <c r="C137">
-        <v>12.262876369845291</v>
+        <v>20.262876369845301</v>
       </c>
       <c r="D137">
-        <v>12.262876369845291</v>
+        <v>22.262876369845301</v>
       </c>
       <c r="E137">
-        <v>12.262876369845291</v>
+        <v>21.262876369845301</v>
       </c>
       <c r="F137">
-        <v>12.262876369845291</v>
+        <v>22.262876369845301</v>
       </c>
       <c r="G137">
-        <v>12.262876369845291</v>
+        <v>21.262876369845301</v>
       </c>
       <c r="H137">
-        <v>12.262876369845291</v>
+        <v>23.262876369845301</v>
       </c>
       <c r="I137">
         <v>22.441505739530559</v>
@@ -8179,7 +8195,7 @@
         <v>21.18899305555556</v>
       </c>
       <c r="M137">
-        <v>-22.893781362007161</v>
+        <v>22.8937813620072</v>
       </c>
       <c r="N137" t="s">
         <v>10</v>
@@ -8193,13 +8209,16 @@
       <c r="Q137">
         <v>6.2649999999999997</v>
       </c>
-    </row>
-    <row r="138" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="R137" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="138" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A138">
         <v>2021</v>
       </c>
       <c r="B138">
-        <v>-69.739769265232979</v>
+        <v>19.739769265233001</v>
       </c>
       <c r="C138">
         <v>22.243313244010562</v>
@@ -8211,16 +8230,16 @@
         <v>22.0298287037037</v>
       </c>
       <c r="F138">
-        <v>20.320004480286741</v>
+        <v>20.320004480286698</v>
       </c>
       <c r="G138">
-        <v>1.7599259259259239</v>
+        <v>21.759925925925899</v>
       </c>
       <c r="H138">
         <v>22.240480997891151</v>
       </c>
       <c r="I138">
-        <v>3.548062519621471</v>
+        <v>23.5480625196214</v>
       </c>
       <c r="J138">
         <v>18.82795601851852</v>
@@ -8246,8 +8265,11 @@
       <c r="Q138">
         <v>6.2649999999999997</v>
       </c>
-    </row>
-    <row r="139" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="R138" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="139" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A139">
         <v>2022</v>
       </c>
@@ -8258,7 +8280,7 @@
         <v>20.699320436507939</v>
       </c>
       <c r="D139">
-        <v>-336.80570179922307</v>
+        <v>16.805701799223002</v>
       </c>
       <c r="E139">
         <v>21.114303240740739</v>
@@ -8267,19 +8289,19 @@
         <v>21.336467293906811</v>
       </c>
       <c r="G139">
-        <v>15.17933564814815</v>
+        <v>25.1793356481482</v>
       </c>
       <c r="H139">
         <v>21.80088485663082</v>
       </c>
       <c r="I139">
-        <v>-15.546105640107429</v>
+        <v>15.546105640107401</v>
       </c>
       <c r="J139">
         <v>20.739831018518519</v>
       </c>
       <c r="K139">
-        <v>6.7894847670250904</v>
+        <v>16.789484767025002</v>
       </c>
       <c r="L139">
         <v>20.376527777777781</v>
@@ -8299,8 +8321,11 @@
       <c r="Q139">
         <v>6.2649999999999997</v>
       </c>
-    </row>
-    <row r="140" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="R139" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="140" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A140">
         <v>2023</v>
       </c>
@@ -8351,6 +8376,9 @@
       </c>
       <c r="Q140">
         <v>6.2649999999999997</v>
+      </c>
+      <c r="R140" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="141" spans="1:18" x14ac:dyDescent="0.35">
@@ -8405,43 +8433,46 @@
       <c r="Q141">
         <v>6.2649999999999997</v>
       </c>
-    </row>
-    <row r="142" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="R141" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="142" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A142">
         <v>2022</v>
       </c>
       <c r="B142">
-        <v>17.04145895118722</v>
+        <v>27.041458951187199</v>
       </c>
       <c r="C142">
-        <v>17.04145895118722</v>
+        <v>25.041458951187199</v>
       </c>
       <c r="D142">
-        <v>17.04145895118722</v>
+        <v>26.041458951187199</v>
       </c>
       <c r="E142">
-        <v>17.04145895118722</v>
+        <v>23.041458951187199</v>
       </c>
       <c r="F142">
-        <v>11.47731917290209</v>
+        <v>23.477319172902099</v>
       </c>
       <c r="G142">
-        <v>17.04145895118722</v>
+        <v>27.041458951187199</v>
       </c>
       <c r="H142">
-        <v>10.59641232492997</v>
+        <v>24.59641232493</v>
       </c>
       <c r="I142">
         <v>21.473210941293441</v>
       </c>
       <c r="J142">
-        <v>17.04145895118722</v>
+        <v>25.041458951187199</v>
       </c>
       <c r="K142">
         <v>20.725484485269408</v>
       </c>
       <c r="L142">
-        <v>17.04145895118722</v>
+        <v>20.041458951187199</v>
       </c>
       <c r="M142">
         <v>20.934867831541219</v>
@@ -8458,8 +8489,11 @@
       <c r="Q142">
         <v>6.2750000000000004</v>
       </c>
-    </row>
-    <row r="143" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="R142" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="143" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A143">
         <v>2023</v>
       </c>
@@ -8510,6 +8544,9 @@
       </c>
       <c r="Q143">
         <v>6.2750000000000004</v>
+      </c>
+      <c r="R143" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="144" spans="1:18" x14ac:dyDescent="0.35">
@@ -8564,9 +8601,17 @@
       <c r="Q144">
         <v>6.2750000000000004</v>
       </c>
+      <c r="R144" t="s">
+        <v>32</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:R144" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="2024"/>
+      </filters>
+    </filterColumn>
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:R144">
       <sortCondition ref="N1:N144"/>
     </sortState>

</xml_diff>